<commit_message>
feat(ui): form polish, unify datatable layout, school profile improvements, remove gender other option, update excel import templates, grading page fixes
</commit_message>
<xml_diff>
--- a/public/templates/students-template.xlsx
+++ b/public/templates/students-template.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Siswa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petunjuk" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +26,65 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEAF1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +92,68 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,56 +519,637 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>nis</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>full_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>gender</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>birth_date</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Contoh Nama Siswa</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>male</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2008-01-15</t>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NIS</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>NISN</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>NIK</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Nama Lengkap</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Jenis Kelamin</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tanggal Lahir</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Tempat Lahir</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Alamat</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Nomor Telepon</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Agama</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Kewarganegaraan</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Anak Ke</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Jumlah Saudara</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Tanggal Masuk</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Asal Sekolah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2024001</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>0012345678</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>3578012345670001</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Ahmad Fauzi</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>2010-05-15</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Surabaya</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Jl. Merdeka No. 10</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>08123456789</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Islam</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>WNI</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>2024-07-15</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>SDN Merdeka 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>← Masukkan data mulai dari baris ini</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Kolom</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Wajib</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Format / Pilihan</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Contoh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>NIS</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Nomor Induk Siswa (unik per sekolah)</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>2024001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>NISN</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Nomor Induk Siswa Nasional</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>0012345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>NIK</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Nomor Induk Kependudukan (16 digit)</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>3578012345670001</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Nama Lengkap</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Nama lengkap siswa tanpa singkatan</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Ahmad Fauzi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Jenis Kelamin</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Jenis kelamin siswa</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>L atau P</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Tanggal Lahir</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Tanggal lahir siswa</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>2010-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Tempat Lahir</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Kota/kabupaten tempat lahir</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Surabaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Alamat</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Alamat tempat tinggal siswa</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Jl. Merdeka No. 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Nomor Telepon</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Nomor HP aktif (siswa atau orang tua)</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>08123456789</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Agama</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Agama yang dianut</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Islam</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Kewarganegaraan</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Status kewarganegaraan</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>WNI</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Anak Ke</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Urutan anak dalam keluarga</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Angka bulat</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Jumlah Saudara</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Jumlah saudara kandung</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Angka bulat</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Tanggal Masuk</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Tanggal pertama masuk sekolah</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>2024-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Asal Sekolah</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Nama sekolah asal (untuk siswa pindahan)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Teks</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>SDN Merdeka 1</t>
         </is>
       </c>
     </row>

</xml_diff>